<commit_message>
test is now good with max decimals
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/thermal_installed_power.xlsx
+++ b/tests/antares/resources/expected_output_files/thermal_installed_power.xlsx
@@ -3658,76 +3658,76 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>2280.990000000001</v>
+        <v>2280.99</v>
       </c>
       <c r="H32" t="n">
-        <v>2280.990000000001</v>
+        <v>2280.99</v>
       </c>
       <c r="I32" t="n">
-        <v>2280.990000000001</v>
+        <v>2280.99</v>
       </c>
       <c r="J32" t="n">
-        <v>2280.990000000001</v>
+        <v>2280.99</v>
       </c>
       <c r="K32" t="n">
-        <v>2280.990000000001</v>
+        <v>2280.99</v>
       </c>
       <c r="L32" t="n">
-        <v>2280.990000000001</v>
+        <v>2280.99</v>
       </c>
       <c r="M32" t="n">
-        <v>2240.990000000001</v>
+        <v>2240.99</v>
       </c>
       <c r="N32" t="n">
-        <v>2240.990000000001</v>
+        <v>2240.99</v>
       </c>
       <c r="O32" t="n">
-        <v>2240.990000000001</v>
+        <v>2240.99</v>
       </c>
       <c r="P32" t="n">
-        <v>2240.990000000001</v>
+        <v>2240.99</v>
       </c>
       <c r="Q32" t="n">
-        <v>2240.990000000001</v>
+        <v>2240.99</v>
       </c>
       <c r="R32" t="n">
-        <v>2240.990000000001</v>
+        <v>2240.99</v>
       </c>
       <c r="S32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="T32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="U32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="V32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="W32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="X32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="Y32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="Z32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="AA32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="AB32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="AC32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="AD32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
     </row>
     <row r="33">
@@ -6106,76 +6106,76 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>109.4886750053054</v>
+        <v>109.489</v>
       </c>
       <c r="H56" t="n">
-        <v>109.4886750053054</v>
+        <v>109.489</v>
       </c>
       <c r="I56" t="n">
-        <v>109.4886750053054</v>
+        <v>109.489</v>
       </c>
       <c r="J56" t="n">
-        <v>109.4886750053054</v>
+        <v>109.489</v>
       </c>
       <c r="K56" t="n">
-        <v>109.4886750053054</v>
+        <v>109.489</v>
       </c>
       <c r="L56" t="n">
-        <v>109.4886750053054</v>
+        <v>109.489</v>
       </c>
       <c r="M56" t="n">
-        <v>122.3886914756762</v>
+        <v>122.389</v>
       </c>
       <c r="N56" t="n">
-        <v>122.3886914756762</v>
+        <v>122.389</v>
       </c>
       <c r="O56" t="n">
-        <v>122.3886914756762</v>
+        <v>122.389</v>
       </c>
       <c r="P56" t="n">
-        <v>122.3886914756762</v>
+        <v>122.389</v>
       </c>
       <c r="Q56" t="n">
-        <v>122.3886914756762</v>
+        <v>122.389</v>
       </c>
       <c r="R56" t="n">
-        <v>122.3886914756762</v>
+        <v>122.389</v>
       </c>
       <c r="S56" t="n">
-        <v>144.3352466512895</v>
+        <v>144.335</v>
       </c>
       <c r="T56" t="n">
-        <v>144.3352466512895</v>
+        <v>144.335</v>
       </c>
       <c r="U56" t="n">
-        <v>144.3352466512895</v>
+        <v>144.335</v>
       </c>
       <c r="V56" t="n">
-        <v>144.3352466512895</v>
+        <v>144.335</v>
       </c>
       <c r="W56" t="n">
-        <v>144.3352466512895</v>
+        <v>144.335</v>
       </c>
       <c r="X56" t="n">
-        <v>144.3352466512895</v>
+        <v>144.335</v>
       </c>
       <c r="Y56" t="n">
-        <v>149.4940714353903</v>
+        <v>149.494</v>
       </c>
       <c r="Z56" t="n">
-        <v>149.4940714353903</v>
+        <v>149.494</v>
       </c>
       <c r="AA56" t="n">
-        <v>149.4940714353903</v>
+        <v>149.494</v>
       </c>
       <c r="AB56" t="n">
-        <v>149.4940714353903</v>
+        <v>149.494</v>
       </c>
       <c r="AC56" t="n">
-        <v>149.4940714353903</v>
+        <v>149.494</v>
       </c>
       <c r="AD56" t="n">
-        <v>149.4940714353903</v>
+        <v>149.494</v>
       </c>
     </row>
     <row r="57">
@@ -6310,76 +6310,76 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>569.9475825619324</v>
+        <v>569.948</v>
       </c>
       <c r="H58" t="n">
-        <v>569.9475825619324</v>
+        <v>569.948</v>
       </c>
       <c r="I58" t="n">
-        <v>569.9475825619324</v>
+        <v>569.948</v>
       </c>
       <c r="J58" t="n">
-        <v>569.9475825619324</v>
+        <v>569.948</v>
       </c>
       <c r="K58" t="n">
-        <v>569.9475825619324</v>
+        <v>569.948</v>
       </c>
       <c r="L58" t="n">
-        <v>569.9475825619324</v>
+        <v>569.948</v>
       </c>
       <c r="M58" t="n">
-        <v>566.5990699412097</v>
+        <v>566.599</v>
       </c>
       <c r="N58" t="n">
-        <v>566.5990699412097</v>
+        <v>566.599</v>
       </c>
       <c r="O58" t="n">
-        <v>566.5990699412097</v>
+        <v>566.599</v>
       </c>
       <c r="P58" t="n">
-        <v>566.5990699412097</v>
+        <v>566.599</v>
       </c>
       <c r="Q58" t="n">
-        <v>566.5990699412097</v>
+        <v>566.599</v>
       </c>
       <c r="R58" t="n">
-        <v>566.5990699412097</v>
+        <v>566.599</v>
       </c>
       <c r="S58" t="n">
-        <v>536.0677170701721</v>
+        <v>536.068</v>
       </c>
       <c r="T58" t="n">
-        <v>536.0677170701721</v>
+        <v>536.068</v>
       </c>
       <c r="U58" t="n">
-        <v>536.0677170701721</v>
+        <v>536.068</v>
       </c>
       <c r="V58" t="n">
-        <v>536.0677170701721</v>
+        <v>536.068</v>
       </c>
       <c r="W58" t="n">
-        <v>536.0677170701721</v>
+        <v>536.068</v>
       </c>
       <c r="X58" t="n">
-        <v>536.0677170701721</v>
+        <v>536.068</v>
       </c>
       <c r="Y58" t="n">
-        <v>523.9241430853729</v>
+        <v>523.924</v>
       </c>
       <c r="Z58" t="n">
-        <v>523.9241430853729</v>
+        <v>523.924</v>
       </c>
       <c r="AA58" t="n">
-        <v>523.9241430853729</v>
+        <v>523.924</v>
       </c>
       <c r="AB58" t="n">
-        <v>523.9241430853729</v>
+        <v>523.924</v>
       </c>
       <c r="AC58" t="n">
-        <v>523.9241430853729</v>
+        <v>523.924</v>
       </c>
       <c r="AD58" t="n">
-        <v>523.9241430853729</v>
+        <v>523.924</v>
       </c>
     </row>
     <row r="59">
@@ -7330,76 +7330,76 @@
         </is>
       </c>
       <c r="G68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="H68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="I68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="J68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="K68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="L68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="M68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="N68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="O68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="P68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="Q68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="R68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="S68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="T68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="U68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="V68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="W68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="X68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="Y68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="Z68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="AA68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="AB68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="AC68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="AD68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
     </row>
     <row r="69">
@@ -8386,40 +8386,40 @@
         <v>733.7</v>
       </c>
       <c r="S78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="T78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="U78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="V78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="W78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="X78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="Y78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="Z78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="AA78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="AB78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="AC78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="AD78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
     </row>
     <row r="79">
@@ -9184,22 +9184,22 @@
         <v>1390.027</v>
       </c>
       <c r="M86" t="n">
-        <v>835.8689999999998</v>
+        <v>835.869</v>
       </c>
       <c r="N86" t="n">
-        <v>835.8689999999998</v>
+        <v>835.869</v>
       </c>
       <c r="O86" t="n">
-        <v>835.8689999999998</v>
+        <v>835.869</v>
       </c>
       <c r="P86" t="n">
-        <v>835.8689999999998</v>
+        <v>835.869</v>
       </c>
       <c r="Q86" t="n">
-        <v>835.8689999999998</v>
+        <v>835.869</v>
       </c>
       <c r="R86" t="n">
-        <v>835.8689999999998</v>
+        <v>835.869</v>
       </c>
       <c r="S86" t="n">
         <v>0</v>
@@ -10186,76 +10186,76 @@
         </is>
       </c>
       <c r="G96" t="n">
-        <v>4840.809999999999</v>
+        <v>4840.81</v>
       </c>
       <c r="H96" t="n">
-        <v>4840.809999999999</v>
+        <v>4840.81</v>
       </c>
       <c r="I96" t="n">
-        <v>4840.809999999999</v>
+        <v>4840.81</v>
       </c>
       <c r="J96" t="n">
-        <v>4840.809999999999</v>
+        <v>4840.81</v>
       </c>
       <c r="K96" t="n">
-        <v>4840.809999999999</v>
+        <v>4840.81</v>
       </c>
       <c r="L96" t="n">
-        <v>4840.809999999999</v>
+        <v>4840.81</v>
       </c>
       <c r="M96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="N96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="O96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="P96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="Q96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="R96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="S96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="T96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="U96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="V96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="W96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="X96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="Y96" t="n">
-        <v>5727.439999999999</v>
+        <v>5727.44</v>
       </c>
       <c r="Z96" t="n">
-        <v>5727.439999999999</v>
+        <v>5727.44</v>
       </c>
       <c r="AA96" t="n">
-        <v>5727.439999999999</v>
+        <v>5727.44</v>
       </c>
       <c r="AB96" t="n">
-        <v>5727.439999999999</v>
+        <v>5727.44</v>
       </c>
       <c r="AC96" t="n">
-        <v>5727.439999999999</v>
+        <v>5727.44</v>
       </c>
       <c r="AD96" t="n">
-        <v>5727.439999999999</v>
+        <v>5727.44</v>
       </c>
     </row>
     <row r="97">
@@ -11038,22 +11038,22 @@
         <v>12217.44</v>
       </c>
       <c r="S104" t="n">
-        <v>8364.300000000001</v>
+        <v>8364.299999999999</v>
       </c>
       <c r="T104" t="n">
-        <v>8364.300000000001</v>
+        <v>8364.299999999999</v>
       </c>
       <c r="U104" t="n">
-        <v>8364.300000000001</v>
+        <v>8364.299999999999</v>
       </c>
       <c r="V104" t="n">
-        <v>8364.300000000001</v>
+        <v>8364.299999999999</v>
       </c>
       <c r="W104" t="n">
-        <v>8364.300000000001</v>
+        <v>8364.299999999999</v>
       </c>
       <c r="X104" t="n">
-        <v>8364.300000000001</v>
+        <v>8364.299999999999</v>
       </c>
       <c r="Y104" t="n">
         <v>4406</v>
@@ -11206,76 +11206,76 @@
         </is>
       </c>
       <c r="G106" t="n">
-        <v>4308.324856428571</v>
+        <v>4308.325</v>
       </c>
       <c r="H106" t="n">
-        <v>4308.324856428571</v>
+        <v>4308.325</v>
       </c>
       <c r="I106" t="n">
-        <v>4308.324856428571</v>
+        <v>4308.325</v>
       </c>
       <c r="J106" t="n">
-        <v>4308.324856428571</v>
+        <v>4308.325</v>
       </c>
       <c r="K106" t="n">
-        <v>4308.324856428571</v>
+        <v>4308.325</v>
       </c>
       <c r="L106" t="n">
-        <v>4308.324856428571</v>
+        <v>4308.325</v>
       </c>
       <c r="M106" t="n">
-        <v>3943.753998571429</v>
+        <v>3943.754</v>
       </c>
       <c r="N106" t="n">
-        <v>3943.753998571429</v>
+        <v>3943.754</v>
       </c>
       <c r="O106" t="n">
-        <v>3943.753998571429</v>
+        <v>3943.754</v>
       </c>
       <c r="P106" t="n">
-        <v>3943.753998571429</v>
+        <v>3943.754</v>
       </c>
       <c r="Q106" t="n">
-        <v>3943.753998571429</v>
+        <v>3943.754</v>
       </c>
       <c r="R106" t="n">
-        <v>3943.753998571429</v>
+        <v>3943.754</v>
       </c>
       <c r="S106" t="n">
-        <v>1668.380120571429</v>
+        <v>1668.38</v>
       </c>
       <c r="T106" t="n">
-        <v>1668.380120571429</v>
+        <v>1668.38</v>
       </c>
       <c r="U106" t="n">
-        <v>1668.380120571429</v>
+        <v>1668.38</v>
       </c>
       <c r="V106" t="n">
-        <v>1668.380120571429</v>
+        <v>1668.38</v>
       </c>
       <c r="W106" t="n">
-        <v>1668.380120571429</v>
+        <v>1668.38</v>
       </c>
       <c r="X106" t="n">
-        <v>1668.380120571429</v>
+        <v>1668.38</v>
       </c>
       <c r="Y106" t="n">
-        <v>964.676164</v>
+        <v>964.676</v>
       </c>
       <c r="Z106" t="n">
-        <v>964.676164</v>
+        <v>964.676</v>
       </c>
       <c r="AA106" t="n">
-        <v>964.676164</v>
+        <v>964.676</v>
       </c>
       <c r="AB106" t="n">
-        <v>964.676164</v>
+        <v>964.676</v>
       </c>
       <c r="AC106" t="n">
-        <v>964.676164</v>
+        <v>964.676</v>
       </c>
       <c r="AD106" t="n">
-        <v>964.676164</v>
+        <v>964.676</v>
       </c>
     </row>
     <row r="107">
@@ -11410,40 +11410,40 @@
         </is>
       </c>
       <c r="G108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="H108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="I108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="J108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="K108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="L108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="M108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="N108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="O108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="P108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="Q108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="R108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="S108" t="n">
         <v>615.15</v>
@@ -12040,22 +12040,22 @@
         <v>1502.55</v>
       </c>
       <c r="M114" t="n">
-        <v>938.5500000000001</v>
+        <v>938.55</v>
       </c>
       <c r="N114" t="n">
-        <v>938.5500000000001</v>
+        <v>938.55</v>
       </c>
       <c r="O114" t="n">
-        <v>938.5500000000001</v>
+        <v>938.55</v>
       </c>
       <c r="P114" t="n">
-        <v>938.5500000000001</v>
+        <v>938.55</v>
       </c>
       <c r="Q114" t="n">
-        <v>938.5500000000001</v>
+        <v>938.55</v>
       </c>
       <c r="R114" t="n">
-        <v>938.5500000000001</v>
+        <v>938.55</v>
       </c>
       <c r="S114" t="n">
         <v>0</v>
@@ -12262,22 +12262,22 @@
         <v>958.42</v>
       </c>
       <c r="S116" t="n">
-        <v>401.1800000000001</v>
+        <v>401.18</v>
       </c>
       <c r="T116" t="n">
-        <v>401.1800000000001</v>
+        <v>401.18</v>
       </c>
       <c r="U116" t="n">
-        <v>401.1800000000001</v>
+        <v>401.18</v>
       </c>
       <c r="V116" t="n">
-        <v>401.1800000000001</v>
+        <v>401.18</v>
       </c>
       <c r="W116" t="n">
-        <v>401.1800000000001</v>
+        <v>401.18</v>
       </c>
       <c r="X116" t="n">
-        <v>401.1800000000001</v>
+        <v>401.18</v>
       </c>
       <c r="Y116" t="n">
         <v>215.78</v>
@@ -12430,31 +12430,31 @@
         </is>
       </c>
       <c r="G118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="H118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="I118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="J118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="K118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="L118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="M118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="N118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="O118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="P118" t="n">
         <v>2398.87</v>
@@ -13450,22 +13450,22 @@
         </is>
       </c>
       <c r="G128" t="n">
-        <v>2771.920000000001</v>
+        <v>2771.92</v>
       </c>
       <c r="H128" t="n">
-        <v>2771.920000000001</v>
+        <v>2771.92</v>
       </c>
       <c r="I128" t="n">
-        <v>2771.920000000001</v>
+        <v>2771.92</v>
       </c>
       <c r="J128" t="n">
-        <v>2771.920000000001</v>
+        <v>2771.92</v>
       </c>
       <c r="K128" t="n">
-        <v>2771.920000000001</v>
+        <v>2771.92</v>
       </c>
       <c r="L128" t="n">
-        <v>2771.920000000001</v>
+        <v>2771.92</v>
       </c>
       <c r="M128" t="n">
         <v>2513.52</v>
@@ -14266,40 +14266,40 @@
         </is>
       </c>
       <c r="G136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="H136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="I136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="J136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="K136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="L136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="M136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="N136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="O136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="P136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="Q136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="R136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="S136" t="n">
         <v>453.84</v>
@@ -15490,76 +15490,76 @@
         </is>
       </c>
       <c r="G148" t="n">
-        <v>125.1726908</v>
+        <v>125.173</v>
       </c>
       <c r="H148" t="n">
-        <v>125.1726908</v>
+        <v>125.173</v>
       </c>
       <c r="I148" t="n">
-        <v>125.1726908</v>
+        <v>125.173</v>
       </c>
       <c r="J148" t="n">
-        <v>125.1726908</v>
+        <v>125.173</v>
       </c>
       <c r="K148" t="n">
-        <v>125.1726908</v>
+        <v>125.173</v>
       </c>
       <c r="L148" t="n">
-        <v>125.1726908</v>
+        <v>125.173</v>
       </c>
       <c r="M148" t="n">
-        <v>115.1120841</v>
+        <v>115.112</v>
       </c>
       <c r="N148" t="n">
-        <v>115.1120841</v>
+        <v>115.112</v>
       </c>
       <c r="O148" t="n">
-        <v>115.1120841</v>
+        <v>115.112</v>
       </c>
       <c r="P148" t="n">
-        <v>115.1120841</v>
+        <v>115.112</v>
       </c>
       <c r="Q148" t="n">
-        <v>115.1120841</v>
+        <v>115.112</v>
       </c>
       <c r="R148" t="n">
-        <v>115.1120841</v>
+        <v>115.112</v>
       </c>
       <c r="S148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="T148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="U148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="V148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="W148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="X148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="Y148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="Z148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="AA148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="AB148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="AC148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="AD148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
     </row>
     <row r="149">
@@ -15694,76 +15694,76 @@
         </is>
       </c>
       <c r="G150" t="n">
-        <v>24.6051092</v>
+        <v>24.605</v>
       </c>
       <c r="H150" t="n">
-        <v>24.6051092</v>
+        <v>24.605</v>
       </c>
       <c r="I150" t="n">
-        <v>24.6051092</v>
+        <v>24.605</v>
       </c>
       <c r="J150" t="n">
-        <v>24.6051092</v>
+        <v>24.605</v>
       </c>
       <c r="K150" t="n">
-        <v>24.6051092</v>
+        <v>24.605</v>
       </c>
       <c r="L150" t="n">
-        <v>24.6051092</v>
+        <v>24.605</v>
       </c>
       <c r="M150" t="n">
-        <v>33.1932159</v>
+        <v>33.193</v>
       </c>
       <c r="N150" t="n">
-        <v>33.1932159</v>
+        <v>33.193</v>
       </c>
       <c r="O150" t="n">
-        <v>33.1932159</v>
+        <v>33.193</v>
       </c>
       <c r="P150" t="n">
-        <v>33.1932159</v>
+        <v>33.193</v>
       </c>
       <c r="Q150" t="n">
-        <v>33.1932159</v>
+        <v>33.193</v>
       </c>
       <c r="R150" t="n">
-        <v>33.1932159</v>
+        <v>33.193</v>
       </c>
       <c r="S150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="T150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="U150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="V150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="W150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="X150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="Y150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="Z150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="AA150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="AB150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="AC150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="AD150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
     </row>
     <row r="151">
@@ -16102,40 +16102,40 @@
         </is>
       </c>
       <c r="G154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="H154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="I154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="J154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="K154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="L154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="M154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="N154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="O154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="P154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="Q154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="R154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="S154" t="n">
         <v>54.3</v>
@@ -16714,76 +16714,76 @@
         </is>
       </c>
       <c r="G160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="H160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="I160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="J160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="K160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="L160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="M160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="N160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="O160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="P160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="Q160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="R160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="S160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="T160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="U160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="V160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="W160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="X160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="Y160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="Z160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="AA160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="AB160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="AC160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="AD160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
     </row>
     <row r="161">
@@ -16918,76 +16918,76 @@
         </is>
       </c>
       <c r="G162" t="n">
-        <v>477.9249</v>
+        <v>477.925</v>
       </c>
       <c r="H162" t="n">
-        <v>477.9249</v>
+        <v>477.925</v>
       </c>
       <c r="I162" t="n">
-        <v>477.9249</v>
+        <v>477.925</v>
       </c>
       <c r="J162" t="n">
-        <v>477.9249</v>
+        <v>477.925</v>
       </c>
       <c r="K162" t="n">
-        <v>477.9249</v>
+        <v>477.925</v>
       </c>
       <c r="L162" t="n">
-        <v>477.9249</v>
+        <v>477.925</v>
       </c>
       <c r="M162" t="n">
-        <v>477.7748999999999</v>
+        <v>477.775</v>
       </c>
       <c r="N162" t="n">
-        <v>477.7748999999999</v>
+        <v>477.775</v>
       </c>
       <c r="O162" t="n">
-        <v>477.7748999999999</v>
+        <v>477.775</v>
       </c>
       <c r="P162" t="n">
-        <v>477.7748999999999</v>
+        <v>477.775</v>
       </c>
       <c r="Q162" t="n">
-        <v>477.7748999999999</v>
+        <v>477.775</v>
       </c>
       <c r="R162" t="n">
-        <v>477.7748999999999</v>
+        <v>477.775</v>
       </c>
       <c r="S162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="T162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="U162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="V162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="W162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="X162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="Y162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="Z162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="AA162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="AB162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="AC162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="AD162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
     </row>
     <row r="163">
@@ -17530,76 +17530,76 @@
         </is>
       </c>
       <c r="G168" t="n">
-        <v>122.5008</v>
+        <v>122.501</v>
       </c>
       <c r="H168" t="n">
-        <v>122.5008</v>
+        <v>122.501</v>
       </c>
       <c r="I168" t="n">
-        <v>122.5008</v>
+        <v>122.501</v>
       </c>
       <c r="J168" t="n">
-        <v>122.5008</v>
+        <v>122.501</v>
       </c>
       <c r="K168" t="n">
-        <v>122.5008</v>
+        <v>122.501</v>
       </c>
       <c r="L168" t="n">
-        <v>122.5008</v>
+        <v>122.501</v>
       </c>
       <c r="M168" t="n">
-        <v>85.9248</v>
+        <v>85.925</v>
       </c>
       <c r="N168" t="n">
-        <v>85.9248</v>
+        <v>85.925</v>
       </c>
       <c r="O168" t="n">
-        <v>85.9248</v>
+        <v>85.925</v>
       </c>
       <c r="P168" t="n">
-        <v>85.9248</v>
+        <v>85.925</v>
       </c>
       <c r="Q168" t="n">
-        <v>85.9248</v>
+        <v>85.925</v>
       </c>
       <c r="R168" t="n">
-        <v>85.9248</v>
+        <v>85.925</v>
       </c>
       <c r="S168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="T168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="U168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="V168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="W168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="X168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="Y168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="Z168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="AA168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="AB168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="AC168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="AD168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
     </row>
     <row r="169">
@@ -17770,40 +17770,40 @@
         <v>56.977</v>
       </c>
       <c r="S170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="T170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="U170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="V170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="W170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="X170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="Y170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="Z170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="AA170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="AB170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="AC170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="AD170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
     </row>
     <row r="171">
@@ -17938,76 +17938,76 @@
         </is>
       </c>
       <c r="G172" t="n">
-        <v>51.91350829040319</v>
+        <v>51.914</v>
       </c>
       <c r="H172" t="n">
-        <v>51.91350829040319</v>
+        <v>51.914</v>
       </c>
       <c r="I172" t="n">
-        <v>51.91350829040319</v>
+        <v>51.914</v>
       </c>
       <c r="J172" t="n">
-        <v>51.91350829040319</v>
+        <v>51.914</v>
       </c>
       <c r="K172" t="n">
-        <v>51.91350829040319</v>
+        <v>51.914</v>
       </c>
       <c r="L172" t="n">
-        <v>51.91350829040319</v>
+        <v>51.914</v>
       </c>
       <c r="M172" t="n">
-        <v>50.91350829040319</v>
+        <v>50.914</v>
       </c>
       <c r="N172" t="n">
-        <v>50.91350829040319</v>
+        <v>50.914</v>
       </c>
       <c r="O172" t="n">
-        <v>50.91350829040319</v>
+        <v>50.914</v>
       </c>
       <c r="P172" t="n">
-        <v>50.91350829040319</v>
+        <v>50.914</v>
       </c>
       <c r="Q172" t="n">
-        <v>50.91350829040319</v>
+        <v>50.914</v>
       </c>
       <c r="R172" t="n">
-        <v>50.91350829040319</v>
+        <v>50.914</v>
       </c>
       <c r="S172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="T172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="U172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="V172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="W172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="X172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="Y172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="Z172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="AA172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="AB172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="AC172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="AD172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
     </row>
     <row r="173">
@@ -18142,76 +18142,76 @@
         </is>
       </c>
       <c r="G174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="H174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="I174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="J174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="K174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="L174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="M174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="N174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="O174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="P174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="Q174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="R174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="S174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="T174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="U174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="V174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="W174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="X174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="Y174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="Z174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="AA174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="AB174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="AC174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="AD174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
     </row>
     <row r="175">
@@ -19162,76 +19162,76 @@
         </is>
       </c>
       <c r="G184" t="n">
-        <v>4085.45378127909</v>
+        <v>4085.454</v>
       </c>
       <c r="H184" t="n">
-        <v>4085.45378127909</v>
+        <v>4085.454</v>
       </c>
       <c r="I184" t="n">
-        <v>4085.45378127909</v>
+        <v>4085.454</v>
       </c>
       <c r="J184" t="n">
-        <v>4085.45378127909</v>
+        <v>4085.454</v>
       </c>
       <c r="K184" t="n">
-        <v>4085.45378127909</v>
+        <v>4085.454</v>
       </c>
       <c r="L184" t="n">
-        <v>4085.45378127909</v>
+        <v>4085.454</v>
       </c>
       <c r="M184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="N184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="O184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="P184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="Q184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="R184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="S184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="T184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="U184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="V184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="W184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="X184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="Y184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="Z184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="AA184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="AB184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="AC184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="AD184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
     </row>
     <row r="185">
@@ -20653,13 +20653,13 @@
         <v>126</v>
       </c>
       <c r="AB198" t="n">
-        <v>72.00000000000001</v>
+        <v>72</v>
       </c>
       <c r="AC198" t="n">
-        <v>72.00000000000001</v>
+        <v>72</v>
       </c>
       <c r="AD198" t="n">
-        <v>72.00000000000001</v>
+        <v>72</v>
       </c>
     </row>
     <row r="199">
@@ -27136,22 +27136,22 @@
         <v>114</v>
       </c>
       <c r="M262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="N262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="O262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="P262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="Q262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="R262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="S262" t="n">
         <v>49</v>
@@ -27172,22 +27172,22 @@
         <v>49</v>
       </c>
       <c r="Y262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="Z262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="AA262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="AB262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="AC262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="AD262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
     </row>
     <row r="263">
@@ -30586,76 +30586,76 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="H296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="I296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="J296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="K296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="L296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="M296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="N296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="O296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="P296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="Q296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="R296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="S296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="T296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="U296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="V296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="W296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="X296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="Y296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="Z296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="AA296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="AB296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="AC296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="AD296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
     </row>
     <row r="297">
@@ -32830,76 +32830,76 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="H318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="I318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="J318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="K318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="L318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="M318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="N318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="O318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="P318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="Q318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="R318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="S318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="T318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="U318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="V318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="W318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="X318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="Y318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="Z318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="AA318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="AB318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="AC318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="AD318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
     </row>
     <row r="319">
@@ -34666,76 +34666,76 @@
         </is>
       </c>
       <c r="G336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="H336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="I336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="J336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="K336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="L336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="M336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="N336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="O336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="P336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="Q336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="R336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="S336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="T336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="U336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="V336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="W336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="X336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="Y336" t="n">
-        <v>2465.2206</v>
+        <v>2465.221</v>
       </c>
       <c r="Z336" t="n">
-        <v>2465.2206</v>
+        <v>2465.221</v>
       </c>
       <c r="AA336" t="n">
-        <v>2465.2206</v>
+        <v>2465.221</v>
       </c>
       <c r="AB336" t="n">
-        <v>2465.2206</v>
+        <v>2465.221</v>
       </c>
       <c r="AC336" t="n">
-        <v>2465.2206</v>
+        <v>2465.221</v>
       </c>
       <c r="AD336" t="n">
-        <v>2465.2206</v>
+        <v>2465.221</v>
       </c>
     </row>
     <row r="337">
@@ -37930,76 +37930,76 @@
         </is>
       </c>
       <c r="G368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="H368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="I368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="J368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="K368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="L368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="M368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="N368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="O368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="P368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="Q368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="R368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="S368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="T368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="U368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="V368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="W368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="X368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="Y368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="Z368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="AA368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="AB368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="AC368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="AD368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
     </row>
     <row r="369">
@@ -39154,40 +39154,40 @@
         </is>
       </c>
       <c r="G380" t="n">
-        <v>9.688995215311005</v>
+        <v>9.689</v>
       </c>
       <c r="H380" t="n">
-        <v>9.688995215311005</v>
+        <v>9.689</v>
       </c>
       <c r="I380" t="n">
-        <v>9.688995215311005</v>
+        <v>9.689</v>
       </c>
       <c r="J380" t="n">
-        <v>9.688995215311005</v>
+        <v>9.689</v>
       </c>
       <c r="K380" t="n">
-        <v>9.688995215311005</v>
+        <v>9.689</v>
       </c>
       <c r="L380" t="n">
-        <v>9.688995215311005</v>
+        <v>9.689</v>
       </c>
       <c r="M380" t="n">
-        <v>6.45933014354067</v>
+        <v>6.459</v>
       </c>
       <c r="N380" t="n">
-        <v>6.45933014354067</v>
+        <v>6.459</v>
       </c>
       <c r="O380" t="n">
-        <v>6.45933014354067</v>
+        <v>6.459</v>
       </c>
       <c r="P380" t="n">
-        <v>6.45933014354067</v>
+        <v>6.459</v>
       </c>
       <c r="Q380" t="n">
-        <v>6.45933014354067</v>
+        <v>6.459</v>
       </c>
       <c r="R380" t="n">
-        <v>6.45933014354067</v>
+        <v>6.459</v>
       </c>
       <c r="S380" t="n">
         <v>0</v>
@@ -44068,22 +44068,22 @@
         <v>0</v>
       </c>
       <c r="M428" t="n">
-        <v>1709.242805870638</v>
+        <v>1709.243</v>
       </c>
       <c r="N428" t="n">
-        <v>1709.242805870638</v>
+        <v>1709.243</v>
       </c>
       <c r="O428" t="n">
-        <v>1709.242805870638</v>
+        <v>1709.243</v>
       </c>
       <c r="P428" t="n">
-        <v>1709.242805870638</v>
+        <v>1709.243</v>
       </c>
       <c r="Q428" t="n">
-        <v>1709.242805870638</v>
+        <v>1709.243</v>
       </c>
       <c r="R428" t="n">
-        <v>1709.242805870638</v>
+        <v>1709.243</v>
       </c>
       <c r="S428" t="n">
         <v>0</v>
@@ -44104,22 +44104,22 @@
         <v>0</v>
       </c>
       <c r="Y428" t="n">
-        <v>1758.618885870638</v>
+        <v>1758.619</v>
       </c>
       <c r="Z428" t="n">
-        <v>1758.618885870638</v>
+        <v>1758.619</v>
       </c>
       <c r="AA428" t="n">
-        <v>1758.618885870638</v>
+        <v>1758.619</v>
       </c>
       <c r="AB428" t="n">
-        <v>1758.618885870638</v>
+        <v>1758.619</v>
       </c>
       <c r="AC428" t="n">
-        <v>1758.618885870638</v>
+        <v>1758.619</v>
       </c>
       <c r="AD428" t="n">
-        <v>1758.618885870638</v>
+        <v>1758.619</v>
       </c>
     </row>
     <row r="429">
@@ -44272,22 +44272,22 @@
         <v>0</v>
       </c>
       <c r="M430" t="n">
-        <v>606.4468800000001</v>
+        <v>606.447</v>
       </c>
       <c r="N430" t="n">
-        <v>606.4468800000001</v>
+        <v>606.447</v>
       </c>
       <c r="O430" t="n">
-        <v>606.4468800000001</v>
+        <v>606.447</v>
       </c>
       <c r="P430" t="n">
-        <v>606.4468800000001</v>
+        <v>606.447</v>
       </c>
       <c r="Q430" t="n">
-        <v>606.4468800000001</v>
+        <v>606.447</v>
       </c>
       <c r="R430" t="n">
-        <v>606.4468800000001</v>
+        <v>606.447</v>
       </c>
       <c r="S430" t="n">
         <v>0</v>
@@ -44308,22 +44308,22 @@
         <v>0</v>
       </c>
       <c r="Y430" t="n">
-        <v>582.4808800000001</v>
+        <v>582.481</v>
       </c>
       <c r="Z430" t="n">
-        <v>582.4808800000001</v>
+        <v>582.481</v>
       </c>
       <c r="AA430" t="n">
-        <v>582.4808800000001</v>
+        <v>582.481</v>
       </c>
       <c r="AB430" t="n">
-        <v>582.4808800000001</v>
+        <v>582.481</v>
       </c>
       <c r="AC430" t="n">
-        <v>582.4808800000001</v>
+        <v>582.481</v>
       </c>
       <c r="AD430" t="n">
-        <v>582.4808800000001</v>
+        <v>582.481</v>
       </c>
     </row>
     <row r="431">
@@ -44662,40 +44662,40 @@
         </is>
       </c>
       <c r="G434" t="n">
-        <v>1984.6245</v>
+        <v>1984.624</v>
       </c>
       <c r="H434" t="n">
-        <v>1984.6245</v>
+        <v>1984.624</v>
       </c>
       <c r="I434" t="n">
-        <v>1984.6245</v>
+        <v>1984.624</v>
       </c>
       <c r="J434" t="n">
-        <v>1984.6245</v>
+        <v>1984.624</v>
       </c>
       <c r="K434" t="n">
-        <v>1984.6245</v>
+        <v>1984.624</v>
       </c>
       <c r="L434" t="n">
-        <v>1984.6245</v>
+        <v>1984.624</v>
       </c>
       <c r="M434" t="n">
-        <v>5100.76803089044</v>
+        <v>5100.768</v>
       </c>
       <c r="N434" t="n">
-        <v>5100.76803089044</v>
+        <v>5100.768</v>
       </c>
       <c r="O434" t="n">
-        <v>5100.76803089044</v>
+        <v>5100.768</v>
       </c>
       <c r="P434" t="n">
-        <v>5100.76803089044</v>
+        <v>5100.768</v>
       </c>
       <c r="Q434" t="n">
-        <v>5100.76803089044</v>
+        <v>5100.768</v>
       </c>
       <c r="R434" t="n">
-        <v>5100.76803089044</v>
+        <v>5100.768</v>
       </c>
       <c r="S434" t="n">
         <v>835</v>
@@ -44716,22 +44716,22 @@
         <v>835</v>
       </c>
       <c r="Y434" t="n">
-        <v>2361.74353089044</v>
+        <v>2361.744</v>
       </c>
       <c r="Z434" t="n">
-        <v>2361.74353089044</v>
+        <v>2361.744</v>
       </c>
       <c r="AA434" t="n">
-        <v>2361.74353089044</v>
+        <v>2361.744</v>
       </c>
       <c r="AB434" t="n">
-        <v>2361.74353089044</v>
+        <v>2361.744</v>
       </c>
       <c r="AC434" t="n">
-        <v>2361.74353089044</v>
+        <v>2361.744</v>
       </c>
       <c r="AD434" t="n">
-        <v>2361.74353089044</v>
+        <v>2361.744</v>
       </c>
     </row>
     <row r="435">
@@ -44866,40 +44866,40 @@
         </is>
       </c>
       <c r="G436" t="n">
-        <v>66.4755</v>
+        <v>66.476</v>
       </c>
       <c r="H436" t="n">
-        <v>66.4755</v>
+        <v>66.476</v>
       </c>
       <c r="I436" t="n">
-        <v>66.4755</v>
+        <v>66.476</v>
       </c>
       <c r="J436" t="n">
-        <v>66.4755</v>
+        <v>66.476</v>
       </c>
       <c r="K436" t="n">
-        <v>66.4755</v>
+        <v>66.476</v>
       </c>
       <c r="L436" t="n">
-        <v>66.4755</v>
+        <v>66.476</v>
       </c>
       <c r="M436" t="n">
-        <v>66.4755</v>
+        <v>66.476</v>
       </c>
       <c r="N436" t="n">
-        <v>66.4755</v>
+        <v>66.476</v>
       </c>
       <c r="O436" t="n">
-        <v>66.4755</v>
+        <v>66.476</v>
       </c>
       <c r="P436" t="n">
-        <v>66.4755</v>
+        <v>66.476</v>
       </c>
       <c r="Q436" t="n">
-        <v>66.4755</v>
+        <v>66.476</v>
       </c>
       <c r="R436" t="n">
-        <v>66.4755</v>
+        <v>66.476</v>
       </c>
       <c r="S436" t="n">
         <v>0</v>
@@ -45070,40 +45070,40 @@
         </is>
       </c>
       <c r="G438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="H438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="I438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="J438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="K438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="L438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="M438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="N438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="O438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="P438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="Q438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="R438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="S438" t="n">
         <v>3670.75</v>
@@ -45274,58 +45274,58 @@
         </is>
       </c>
       <c r="G440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="H440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="I440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="J440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="K440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="L440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="M440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="N440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="O440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="P440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="Q440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="R440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="S440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="T440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="U440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="V440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="W440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="X440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="Y440" t="n">
         <v>0</v>
@@ -50170,76 +50170,76 @@
         </is>
       </c>
       <c r="G488" t="n">
-        <v>212.148282494181</v>
+        <v>212.148</v>
       </c>
       <c r="H488" t="n">
-        <v>212.148282494181</v>
+        <v>212.148</v>
       </c>
       <c r="I488" t="n">
-        <v>212.148282494181</v>
+        <v>212.148</v>
       </c>
       <c r="J488" t="n">
-        <v>212.148282494181</v>
+        <v>212.148</v>
       </c>
       <c r="K488" t="n">
-        <v>212.148282494181</v>
+        <v>212.148</v>
       </c>
       <c r="L488" t="n">
-        <v>218.5108942790641</v>
+        <v>218.511</v>
       </c>
       <c r="M488" t="n">
-        <v>218.5108942790641</v>
+        <v>218.511</v>
       </c>
       <c r="N488" t="n">
-        <v>218.5108942790641</v>
+        <v>218.511</v>
       </c>
       <c r="O488" t="n">
-        <v>218.5108942790641</v>
+        <v>218.511</v>
       </c>
       <c r="P488" t="n">
-        <v>218.5108942790641</v>
+        <v>218.511</v>
       </c>
       <c r="Q488" t="n">
-        <v>218.5108942790641</v>
+        <v>218.511</v>
       </c>
       <c r="R488" t="n">
-        <v>218.5108942790641</v>
+        <v>218.511</v>
       </c>
       <c r="S488" t="n">
-        <v>242.2384454244763</v>
+        <v>242.238</v>
       </c>
       <c r="T488" t="n">
-        <v>242.2384454244763</v>
+        <v>242.238</v>
       </c>
       <c r="U488" t="n">
-        <v>242.2384454244763</v>
+        <v>242.238</v>
       </c>
       <c r="V488" t="n">
-        <v>242.2384454244763</v>
+        <v>242.238</v>
       </c>
       <c r="W488" t="n">
-        <v>242.2384454244763</v>
+        <v>242.238</v>
       </c>
       <c r="X488" t="n">
-        <v>248.0267585446527</v>
+        <v>248.027</v>
       </c>
       <c r="Y488" t="n">
-        <v>248.0267585446527</v>
+        <v>248.027</v>
       </c>
       <c r="Z488" t="n">
-        <v>248.0267585446527</v>
+        <v>248.027</v>
       </c>
       <c r="AA488" t="n">
-        <v>248.0267585446527</v>
+        <v>248.027</v>
       </c>
       <c r="AB488" t="n">
-        <v>248.0267585446527</v>
+        <v>248.027</v>
       </c>
       <c r="AC488" t="n">
-        <v>248.0267585446527</v>
+        <v>248.027</v>
       </c>
       <c r="AD488" t="n">
-        <v>248.0267585446527</v>
+        <v>248.027</v>
       </c>
     </row>
     <row r="489">
@@ -51598,76 +51598,76 @@
         </is>
       </c>
       <c r="G502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="H502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="I502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="J502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="K502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="L502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="M502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="N502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="O502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="P502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="Q502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="R502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="S502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="T502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="U502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="V502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="W502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="X502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="Y502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="Z502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="AA502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="AB502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="AC502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="AD502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
     </row>
     <row r="503">
@@ -51802,76 +51802,76 @@
         </is>
       </c>
       <c r="G504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="H504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="I504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="J504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="K504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="L504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="M504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="N504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="O504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="P504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="Q504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="R504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="S504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="T504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="U504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="V504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="W504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="X504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="Y504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="Z504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="AA504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="AB504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="AC504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="AD504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
     </row>
     <row r="505">
@@ -52006,76 +52006,76 @@
         </is>
       </c>
       <c r="G506" t="n">
-        <v>120.8717305699482</v>
+        <v>120.872</v>
       </c>
       <c r="H506" t="n">
-        <v>120.8717305699482</v>
+        <v>120.872</v>
       </c>
       <c r="I506" t="n">
-        <v>120.8717305699482</v>
+        <v>120.872</v>
       </c>
       <c r="J506" t="n">
-        <v>120.8717305699482</v>
+        <v>120.872</v>
       </c>
       <c r="K506" t="n">
-        <v>120.8717305699482</v>
+        <v>120.872</v>
       </c>
       <c r="L506" t="n">
-        <v>120.8717305699482</v>
+        <v>120.872</v>
       </c>
       <c r="M506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="N506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="O506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="P506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="Q506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="R506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="S506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="T506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="U506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="V506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="W506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="X506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="Y506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="Z506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="AA506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="AB506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="AC506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="AD506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
     </row>
     <row r="507">
@@ -53026,76 +53026,76 @@
         </is>
       </c>
       <c r="G516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="H516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="I516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="J516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="K516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="L516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="M516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="N516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="O516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="P516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="Q516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="R516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="S516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="T516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="U516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="V516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="W516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="X516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="Y516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="Z516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="AA516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="AB516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="AC516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="AD516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
     </row>
     <row r="517">
@@ -53230,76 +53230,76 @@
         </is>
       </c>
       <c r="G518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="H518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="I518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="J518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="K518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="L518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="M518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="N518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="O518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="P518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="Q518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="R518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="S518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="T518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="U518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="V518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="W518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="X518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="Y518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="Z518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="AA518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="AB518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="AC518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="AD518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="519">
@@ -53638,76 +53638,76 @@
         </is>
       </c>
       <c r="G522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="H522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="I522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="J522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="K522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="L522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="M522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="N522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="O522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="P522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="Q522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="R522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="S522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="T522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="U522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="V522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="W522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="X522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="Y522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="Z522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="AA522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="AB522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="AC522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="AD522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
     </row>
     <row r="523">
@@ -53842,76 +53842,76 @@
         </is>
       </c>
       <c r="G524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="H524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="I524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="J524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="K524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="L524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="M524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="N524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="O524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="P524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="Q524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="R524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="S524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="T524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="U524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="V524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="W524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="X524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="Y524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="Z524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="AA524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="AB524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="AC524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="AD524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
     </row>
     <row r="525">
@@ -54250,76 +54250,76 @@
         </is>
       </c>
       <c r="G528" t="n">
-        <v>2789.137264415848</v>
+        <v>2789.137</v>
       </c>
       <c r="H528" t="n">
-        <v>2789.137264415848</v>
+        <v>2789.137</v>
       </c>
       <c r="I528" t="n">
-        <v>2789.137264415848</v>
+        <v>2789.137</v>
       </c>
       <c r="J528" t="n">
-        <v>2789.137264415848</v>
+        <v>2789.137</v>
       </c>
       <c r="K528" t="n">
-        <v>2789.137264415848</v>
+        <v>2789.137</v>
       </c>
       <c r="L528" t="n">
-        <v>2789.137264415848</v>
+        <v>2789.137</v>
       </c>
       <c r="M528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="N528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="O528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="P528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="Q528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="R528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="S528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="T528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="U528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="V528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="W528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="X528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="Y528" t="n">
-        <v>2829.637264415848</v>
+        <v>2829.637</v>
       </c>
       <c r="Z528" t="n">
-        <v>2829.637264415848</v>
+        <v>2829.637</v>
       </c>
       <c r="AA528" t="n">
-        <v>2829.637264415848</v>
+        <v>2829.637</v>
       </c>
       <c r="AB528" t="n">
-        <v>2829.637264415848</v>
+        <v>2829.637</v>
       </c>
       <c r="AC528" t="n">
-        <v>2829.637264415848</v>
+        <v>2829.637</v>
       </c>
       <c r="AD528" t="n">
-        <v>2829.637264415848</v>
+        <v>2829.637</v>
       </c>
     </row>
     <row r="529">
@@ -55120,22 +55120,22 @@
         <v>1612.71</v>
       </c>
       <c r="Y536" t="n">
-        <v>851.0699999999999</v>
+        <v>851.0700000000001</v>
       </c>
       <c r="Z536" t="n">
-        <v>851.0699999999999</v>
+        <v>851.0700000000001</v>
       </c>
       <c r="AA536" t="n">
-        <v>851.0699999999999</v>
+        <v>851.0700000000001</v>
       </c>
       <c r="AB536" t="n">
-        <v>851.0699999999999</v>
+        <v>851.0700000000001</v>
       </c>
       <c r="AC536" t="n">
-        <v>851.0699999999999</v>
+        <v>851.0700000000001</v>
       </c>
       <c r="AD536" t="n">
-        <v>851.0699999999999</v>
+        <v>851.0700000000001</v>
       </c>
     </row>
     <row r="537">

</xml_diff>

<commit_message>
perf(install power): various modifications (#39)
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/thermal_installed_power.xlsx
+++ b/tests/antares/resources/expected_output_files/thermal_installed_power.xlsx
@@ -616,7 +616,7 @@
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="N2" t="n">
         <v>200</v>
@@ -718,7 +718,7 @@
         <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
         <v>2</v>
@@ -3658,76 +3658,76 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>2280.990000000001</v>
+        <v>2280.99</v>
       </c>
       <c r="H32" t="n">
-        <v>2280.990000000001</v>
+        <v>2280.99</v>
       </c>
       <c r="I32" t="n">
-        <v>2280.990000000001</v>
+        <v>2280.99</v>
       </c>
       <c r="J32" t="n">
-        <v>2280.990000000001</v>
+        <v>2280.99</v>
       </c>
       <c r="K32" t="n">
-        <v>2280.990000000001</v>
+        <v>2280.99</v>
       </c>
       <c r="L32" t="n">
-        <v>2280.990000000001</v>
+        <v>2280.99</v>
       </c>
       <c r="M32" t="n">
-        <v>2240.990000000001</v>
+        <v>2240.99</v>
       </c>
       <c r="N32" t="n">
-        <v>2240.990000000001</v>
+        <v>2240.99</v>
       </c>
       <c r="O32" t="n">
-        <v>2240.990000000001</v>
+        <v>2240.99</v>
       </c>
       <c r="P32" t="n">
-        <v>2240.990000000001</v>
+        <v>2240.99</v>
       </c>
       <c r="Q32" t="n">
-        <v>2240.990000000001</v>
+        <v>2240.99</v>
       </c>
       <c r="R32" t="n">
-        <v>2240.990000000001</v>
+        <v>2240.99</v>
       </c>
       <c r="S32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="T32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="U32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="V32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="W32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="X32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="Y32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="Z32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="AA32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="AB32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="AC32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
       <c r="AD32" t="n">
-        <v>2210.990000000001</v>
+        <v>2210.99</v>
       </c>
     </row>
     <row r="33">
@@ -6106,76 +6106,76 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>109.4886750053054</v>
+        <v>109.489</v>
       </c>
       <c r="H56" t="n">
-        <v>109.4886750053054</v>
+        <v>109.489</v>
       </c>
       <c r="I56" t="n">
-        <v>109.4886750053054</v>
+        <v>109.489</v>
       </c>
       <c r="J56" t="n">
-        <v>109.4886750053054</v>
+        <v>109.489</v>
       </c>
       <c r="K56" t="n">
-        <v>109.4886750053054</v>
+        <v>109.489</v>
       </c>
       <c r="L56" t="n">
-        <v>109.4886750053054</v>
+        <v>109.489</v>
       </c>
       <c r="M56" t="n">
-        <v>122.3886914756762</v>
+        <v>122.389</v>
       </c>
       <c r="N56" t="n">
-        <v>122.3886914756762</v>
+        <v>122.389</v>
       </c>
       <c r="O56" t="n">
-        <v>122.3886914756762</v>
+        <v>122.389</v>
       </c>
       <c r="P56" t="n">
-        <v>122.3886914756762</v>
+        <v>122.389</v>
       </c>
       <c r="Q56" t="n">
-        <v>122.3886914756762</v>
+        <v>122.389</v>
       </c>
       <c r="R56" t="n">
-        <v>122.3886914756762</v>
+        <v>122.389</v>
       </c>
       <c r="S56" t="n">
-        <v>144.3352466512895</v>
+        <v>144.335</v>
       </c>
       <c r="T56" t="n">
-        <v>144.3352466512895</v>
+        <v>144.335</v>
       </c>
       <c r="U56" t="n">
-        <v>144.3352466512895</v>
+        <v>144.335</v>
       </c>
       <c r="V56" t="n">
-        <v>144.3352466512895</v>
+        <v>144.335</v>
       </c>
       <c r="W56" t="n">
-        <v>144.3352466512895</v>
+        <v>144.335</v>
       </c>
       <c r="X56" t="n">
-        <v>144.3352466512895</v>
+        <v>144.335</v>
       </c>
       <c r="Y56" t="n">
-        <v>149.4940714353903</v>
+        <v>149.494</v>
       </c>
       <c r="Z56" t="n">
-        <v>149.4940714353903</v>
+        <v>149.494</v>
       </c>
       <c r="AA56" t="n">
-        <v>149.4940714353903</v>
+        <v>149.494</v>
       </c>
       <c r="AB56" t="n">
-        <v>149.4940714353903</v>
+        <v>149.494</v>
       </c>
       <c r="AC56" t="n">
-        <v>149.4940714353903</v>
+        <v>149.494</v>
       </c>
       <c r="AD56" t="n">
-        <v>149.4940714353903</v>
+        <v>149.494</v>
       </c>
     </row>
     <row r="57">
@@ -6310,76 +6310,76 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>569.9475825619324</v>
+        <v>569.948</v>
       </c>
       <c r="H58" t="n">
-        <v>569.9475825619324</v>
+        <v>569.948</v>
       </c>
       <c r="I58" t="n">
-        <v>569.9475825619324</v>
+        <v>569.948</v>
       </c>
       <c r="J58" t="n">
-        <v>569.9475825619324</v>
+        <v>569.948</v>
       </c>
       <c r="K58" t="n">
-        <v>569.9475825619324</v>
+        <v>569.948</v>
       </c>
       <c r="L58" t="n">
-        <v>569.9475825619324</v>
+        <v>569.948</v>
       </c>
       <c r="M58" t="n">
-        <v>566.5990699412097</v>
+        <v>566.599</v>
       </c>
       <c r="N58" t="n">
-        <v>566.5990699412097</v>
+        <v>566.599</v>
       </c>
       <c r="O58" t="n">
-        <v>566.5990699412097</v>
+        <v>566.599</v>
       </c>
       <c r="P58" t="n">
-        <v>566.5990699412097</v>
+        <v>566.599</v>
       </c>
       <c r="Q58" t="n">
-        <v>566.5990699412097</v>
+        <v>566.599</v>
       </c>
       <c r="R58" t="n">
-        <v>566.5990699412097</v>
+        <v>566.599</v>
       </c>
       <c r="S58" t="n">
-        <v>536.0677170701721</v>
+        <v>536.068</v>
       </c>
       <c r="T58" t="n">
-        <v>536.0677170701721</v>
+        <v>536.068</v>
       </c>
       <c r="U58" t="n">
-        <v>536.0677170701721</v>
+        <v>536.068</v>
       </c>
       <c r="V58" t="n">
-        <v>536.0677170701721</v>
+        <v>536.068</v>
       </c>
       <c r="W58" t="n">
-        <v>536.0677170701721</v>
+        <v>536.068</v>
       </c>
       <c r="X58" t="n">
-        <v>536.0677170701721</v>
+        <v>536.068</v>
       </c>
       <c r="Y58" t="n">
-        <v>523.9241430853729</v>
+        <v>523.924</v>
       </c>
       <c r="Z58" t="n">
-        <v>523.9241430853729</v>
+        <v>523.924</v>
       </c>
       <c r="AA58" t="n">
-        <v>523.9241430853729</v>
+        <v>523.924</v>
       </c>
       <c r="AB58" t="n">
-        <v>523.9241430853729</v>
+        <v>523.924</v>
       </c>
       <c r="AC58" t="n">
-        <v>523.9241430853729</v>
+        <v>523.924</v>
       </c>
       <c r="AD58" t="n">
-        <v>523.9241430853729</v>
+        <v>523.924</v>
       </c>
     </row>
     <row r="59">
@@ -7330,76 +7330,76 @@
         </is>
       </c>
       <c r="G68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="H68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="I68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="J68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="K68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="L68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="M68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="N68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="O68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="P68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="Q68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="R68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="S68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="T68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="U68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="V68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="W68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="X68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="Y68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="Z68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="AA68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="AB68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="AC68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
       <c r="AD68" t="n">
-        <v>16.26333333333334</v>
+        <v>16.263</v>
       </c>
     </row>
     <row r="69">
@@ -8386,40 +8386,40 @@
         <v>733.7</v>
       </c>
       <c r="S78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="T78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="U78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="V78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="W78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="X78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="Y78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="Z78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="AA78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="AB78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="AC78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
       <c r="AD78" t="n">
-        <v>794.8100000000001</v>
+        <v>794.8099999999999</v>
       </c>
     </row>
     <row r="79">
@@ -9184,22 +9184,22 @@
         <v>1390.027</v>
       </c>
       <c r="M86" t="n">
-        <v>835.8689999999998</v>
+        <v>835.869</v>
       </c>
       <c r="N86" t="n">
-        <v>835.8689999999998</v>
+        <v>835.869</v>
       </c>
       <c r="O86" t="n">
-        <v>835.8689999999998</v>
+        <v>835.869</v>
       </c>
       <c r="P86" t="n">
-        <v>835.8689999999998</v>
+        <v>835.869</v>
       </c>
       <c r="Q86" t="n">
-        <v>835.8689999999998</v>
+        <v>835.869</v>
       </c>
       <c r="R86" t="n">
-        <v>835.8689999999998</v>
+        <v>835.869</v>
       </c>
       <c r="S86" t="n">
         <v>0</v>
@@ -10186,76 +10186,76 @@
         </is>
       </c>
       <c r="G96" t="n">
-        <v>4840.809999999999</v>
+        <v>4840.81</v>
       </c>
       <c r="H96" t="n">
-        <v>4840.809999999999</v>
+        <v>4840.81</v>
       </c>
       <c r="I96" t="n">
-        <v>4840.809999999999</v>
+        <v>4840.81</v>
       </c>
       <c r="J96" t="n">
-        <v>4840.809999999999</v>
+        <v>4840.81</v>
       </c>
       <c r="K96" t="n">
-        <v>4840.809999999999</v>
+        <v>4840.81</v>
       </c>
       <c r="L96" t="n">
-        <v>4840.809999999999</v>
+        <v>4840.81</v>
       </c>
       <c r="M96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="N96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="O96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="P96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="Q96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="R96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="S96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="T96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="U96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="V96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="W96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="X96" t="n">
-        <v>5875.809999999999</v>
+        <v>5875.81</v>
       </c>
       <c r="Y96" t="n">
-        <v>5727.439999999999</v>
+        <v>5727.44</v>
       </c>
       <c r="Z96" t="n">
-        <v>5727.439999999999</v>
+        <v>5727.44</v>
       </c>
       <c r="AA96" t="n">
-        <v>5727.439999999999</v>
+        <v>5727.44</v>
       </c>
       <c r="AB96" t="n">
-        <v>5727.439999999999</v>
+        <v>5727.44</v>
       </c>
       <c r="AC96" t="n">
-        <v>5727.439999999999</v>
+        <v>5727.44</v>
       </c>
       <c r="AD96" t="n">
-        <v>5727.439999999999</v>
+        <v>5727.44</v>
       </c>
     </row>
     <row r="97">
@@ -11038,22 +11038,22 @@
         <v>12217.44</v>
       </c>
       <c r="S104" t="n">
-        <v>8364.300000000001</v>
+        <v>8364.299999999999</v>
       </c>
       <c r="T104" t="n">
-        <v>8364.300000000001</v>
+        <v>8364.299999999999</v>
       </c>
       <c r="U104" t="n">
-        <v>8364.300000000001</v>
+        <v>8364.299999999999</v>
       </c>
       <c r="V104" t="n">
-        <v>8364.300000000001</v>
+        <v>8364.299999999999</v>
       </c>
       <c r="W104" t="n">
-        <v>8364.300000000001</v>
+        <v>8364.299999999999</v>
       </c>
       <c r="X104" t="n">
-        <v>8364.300000000001</v>
+        <v>8364.299999999999</v>
       </c>
       <c r="Y104" t="n">
         <v>4406</v>
@@ -11206,76 +11206,76 @@
         </is>
       </c>
       <c r="G106" t="n">
-        <v>4308.324856428571</v>
+        <v>4308.325</v>
       </c>
       <c r="H106" t="n">
-        <v>4308.324856428571</v>
+        <v>4308.325</v>
       </c>
       <c r="I106" t="n">
-        <v>4308.324856428571</v>
+        <v>4308.325</v>
       </c>
       <c r="J106" t="n">
-        <v>4308.324856428571</v>
+        <v>4308.325</v>
       </c>
       <c r="K106" t="n">
-        <v>4308.324856428571</v>
+        <v>4308.325</v>
       </c>
       <c r="L106" t="n">
-        <v>4308.324856428571</v>
+        <v>4308.325</v>
       </c>
       <c r="M106" t="n">
-        <v>3943.753998571429</v>
+        <v>3943.754</v>
       </c>
       <c r="N106" t="n">
-        <v>3943.753998571429</v>
+        <v>3943.754</v>
       </c>
       <c r="O106" t="n">
-        <v>3943.753998571429</v>
+        <v>3943.754</v>
       </c>
       <c r="P106" t="n">
-        <v>3943.753998571429</v>
+        <v>3943.754</v>
       </c>
       <c r="Q106" t="n">
-        <v>3943.753998571429</v>
+        <v>3943.754</v>
       </c>
       <c r="R106" t="n">
-        <v>3943.753998571429</v>
+        <v>3943.754</v>
       </c>
       <c r="S106" t="n">
-        <v>1668.380120571429</v>
+        <v>1668.38</v>
       </c>
       <c r="T106" t="n">
-        <v>1668.380120571429</v>
+        <v>1668.38</v>
       </c>
       <c r="U106" t="n">
-        <v>1668.380120571429</v>
+        <v>1668.38</v>
       </c>
       <c r="V106" t="n">
-        <v>1668.380120571429</v>
+        <v>1668.38</v>
       </c>
       <c r="W106" t="n">
-        <v>1668.380120571429</v>
+        <v>1668.38</v>
       </c>
       <c r="X106" t="n">
-        <v>1668.380120571429</v>
+        <v>1668.38</v>
       </c>
       <c r="Y106" t="n">
-        <v>964.676164</v>
+        <v>964.676</v>
       </c>
       <c r="Z106" t="n">
-        <v>964.676164</v>
+        <v>964.676</v>
       </c>
       <c r="AA106" t="n">
-        <v>964.676164</v>
+        <v>964.676</v>
       </c>
       <c r="AB106" t="n">
-        <v>964.676164</v>
+        <v>964.676</v>
       </c>
       <c r="AC106" t="n">
-        <v>964.676164</v>
+        <v>964.676</v>
       </c>
       <c r="AD106" t="n">
-        <v>964.676164</v>
+        <v>964.676</v>
       </c>
     </row>
     <row r="107">
@@ -11410,40 +11410,40 @@
         </is>
       </c>
       <c r="G108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="H108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="I108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="J108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="K108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="L108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="M108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="N108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="O108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="P108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="Q108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="R108" t="n">
-        <v>747.1999999999999</v>
+        <v>747.2</v>
       </c>
       <c r="S108" t="n">
         <v>615.15</v>
@@ -12040,22 +12040,22 @@
         <v>1502.55</v>
       </c>
       <c r="M114" t="n">
-        <v>938.5500000000001</v>
+        <v>938.55</v>
       </c>
       <c r="N114" t="n">
-        <v>938.5500000000001</v>
+        <v>938.55</v>
       </c>
       <c r="O114" t="n">
-        <v>938.5500000000001</v>
+        <v>938.55</v>
       </c>
       <c r="P114" t="n">
-        <v>938.5500000000001</v>
+        <v>938.55</v>
       </c>
       <c r="Q114" t="n">
-        <v>938.5500000000001</v>
+        <v>938.55</v>
       </c>
       <c r="R114" t="n">
-        <v>938.5500000000001</v>
+        <v>938.55</v>
       </c>
       <c r="S114" t="n">
         <v>0</v>
@@ -12262,22 +12262,22 @@
         <v>958.42</v>
       </c>
       <c r="S116" t="n">
-        <v>401.1800000000001</v>
+        <v>401.18</v>
       </c>
       <c r="T116" t="n">
-        <v>401.1800000000001</v>
+        <v>401.18</v>
       </c>
       <c r="U116" t="n">
-        <v>401.1800000000001</v>
+        <v>401.18</v>
       </c>
       <c r="V116" t="n">
-        <v>401.1800000000001</v>
+        <v>401.18</v>
       </c>
       <c r="W116" t="n">
-        <v>401.1800000000001</v>
+        <v>401.18</v>
       </c>
       <c r="X116" t="n">
-        <v>401.1800000000001</v>
+        <v>401.18</v>
       </c>
       <c r="Y116" t="n">
         <v>215.78</v>
@@ -12430,31 +12430,31 @@
         </is>
       </c>
       <c r="G118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="H118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="I118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="J118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="K118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="L118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="M118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="N118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="O118" t="n">
-        <v>4402.870000000001</v>
+        <v>4402.87</v>
       </c>
       <c r="P118" t="n">
         <v>2398.87</v>
@@ -13450,22 +13450,22 @@
         </is>
       </c>
       <c r="G128" t="n">
-        <v>2771.920000000001</v>
+        <v>2771.92</v>
       </c>
       <c r="H128" t="n">
-        <v>2771.920000000001</v>
+        <v>2771.92</v>
       </c>
       <c r="I128" t="n">
-        <v>2771.920000000001</v>
+        <v>2771.92</v>
       </c>
       <c r="J128" t="n">
-        <v>2771.920000000001</v>
+        <v>2771.92</v>
       </c>
       <c r="K128" t="n">
-        <v>2771.920000000001</v>
+        <v>2771.92</v>
       </c>
       <c r="L128" t="n">
-        <v>2771.920000000001</v>
+        <v>2771.92</v>
       </c>
       <c r="M128" t="n">
         <v>2513.52</v>
@@ -14266,40 +14266,40 @@
         </is>
       </c>
       <c r="G136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="H136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="I136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="J136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="K136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="L136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="M136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="N136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="O136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="P136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="Q136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="R136" t="n">
-        <v>523.8399999999999</v>
+        <v>523.84</v>
       </c>
       <c r="S136" t="n">
         <v>453.84</v>
@@ -15490,76 +15490,76 @@
         </is>
       </c>
       <c r="G148" t="n">
-        <v>125.1726908</v>
+        <v>125.173</v>
       </c>
       <c r="H148" t="n">
-        <v>125.1726908</v>
+        <v>125.173</v>
       </c>
       <c r="I148" t="n">
-        <v>125.1726908</v>
+        <v>125.173</v>
       </c>
       <c r="J148" t="n">
-        <v>125.1726908</v>
+        <v>125.173</v>
       </c>
       <c r="K148" t="n">
-        <v>125.1726908</v>
+        <v>125.173</v>
       </c>
       <c r="L148" t="n">
-        <v>125.1726908</v>
+        <v>125.173</v>
       </c>
       <c r="M148" t="n">
-        <v>115.1120841</v>
+        <v>115.112</v>
       </c>
       <c r="N148" t="n">
-        <v>115.1120841</v>
+        <v>115.112</v>
       </c>
       <c r="O148" t="n">
-        <v>115.1120841</v>
+        <v>115.112</v>
       </c>
       <c r="P148" t="n">
-        <v>115.1120841</v>
+        <v>115.112</v>
       </c>
       <c r="Q148" t="n">
-        <v>115.1120841</v>
+        <v>115.112</v>
       </c>
       <c r="R148" t="n">
-        <v>115.1120841</v>
+        <v>115.112</v>
       </c>
       <c r="S148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="T148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="U148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="V148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="W148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="X148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="Y148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="Z148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="AA148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="AB148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="AC148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
       <c r="AD148" t="n">
-        <v>120.4235511</v>
+        <v>120.424</v>
       </c>
     </row>
     <row r="149">
@@ -15694,76 +15694,76 @@
         </is>
       </c>
       <c r="G150" t="n">
-        <v>24.6051092</v>
+        <v>24.605</v>
       </c>
       <c r="H150" t="n">
-        <v>24.6051092</v>
+        <v>24.605</v>
       </c>
       <c r="I150" t="n">
-        <v>24.6051092</v>
+        <v>24.605</v>
       </c>
       <c r="J150" t="n">
-        <v>24.6051092</v>
+        <v>24.605</v>
       </c>
       <c r="K150" t="n">
-        <v>24.6051092</v>
+        <v>24.605</v>
       </c>
       <c r="L150" t="n">
-        <v>24.6051092</v>
+        <v>24.605</v>
       </c>
       <c r="M150" t="n">
-        <v>33.1932159</v>
+        <v>33.193</v>
       </c>
       <c r="N150" t="n">
-        <v>33.1932159</v>
+        <v>33.193</v>
       </c>
       <c r="O150" t="n">
-        <v>33.1932159</v>
+        <v>33.193</v>
       </c>
       <c r="P150" t="n">
-        <v>33.1932159</v>
+        <v>33.193</v>
       </c>
       <c r="Q150" t="n">
-        <v>33.1932159</v>
+        <v>33.193</v>
       </c>
       <c r="R150" t="n">
-        <v>33.1932159</v>
+        <v>33.193</v>
       </c>
       <c r="S150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="T150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="U150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="V150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="W150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="X150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="Y150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="Z150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="AA150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="AB150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="AC150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
       <c r="AD150" t="n">
-        <v>23.8537489</v>
+        <v>23.854</v>
       </c>
     </row>
     <row r="151">
@@ -16102,40 +16102,40 @@
         </is>
       </c>
       <c r="G154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="H154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="I154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="J154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="K154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="L154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="M154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="N154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="O154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="P154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="Q154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="R154" t="n">
-        <v>107.2884</v>
+        <v>107.288</v>
       </c>
       <c r="S154" t="n">
         <v>54.3</v>
@@ -16714,76 +16714,76 @@
         </is>
       </c>
       <c r="G160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="H160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="I160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="J160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="K160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="L160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="M160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="N160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="O160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="P160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="Q160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="R160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="S160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="T160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="U160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="V160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="W160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="X160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="Y160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="Z160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="AA160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="AB160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="AC160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
       <c r="AD160" t="n">
-        <v>0.9231000000000003</v>
+        <v>0.923</v>
       </c>
     </row>
     <row r="161">
@@ -16918,76 +16918,76 @@
         </is>
       </c>
       <c r="G162" t="n">
-        <v>477.9249</v>
+        <v>477.925</v>
       </c>
       <c r="H162" t="n">
-        <v>477.9249</v>
+        <v>477.925</v>
       </c>
       <c r="I162" t="n">
-        <v>477.9249</v>
+        <v>477.925</v>
       </c>
       <c r="J162" t="n">
-        <v>477.9249</v>
+        <v>477.925</v>
       </c>
       <c r="K162" t="n">
-        <v>477.9249</v>
+        <v>477.925</v>
       </c>
       <c r="L162" t="n">
-        <v>477.9249</v>
+        <v>477.925</v>
       </c>
       <c r="M162" t="n">
-        <v>477.7748999999999</v>
+        <v>477.775</v>
       </c>
       <c r="N162" t="n">
-        <v>477.7748999999999</v>
+        <v>477.775</v>
       </c>
       <c r="O162" t="n">
-        <v>477.7748999999999</v>
+        <v>477.775</v>
       </c>
       <c r="P162" t="n">
-        <v>477.7748999999999</v>
+        <v>477.775</v>
       </c>
       <c r="Q162" t="n">
-        <v>477.7748999999999</v>
+        <v>477.775</v>
       </c>
       <c r="R162" t="n">
-        <v>477.7748999999999</v>
+        <v>477.775</v>
       </c>
       <c r="S162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="T162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="U162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="V162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="W162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="X162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="Y162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="Z162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="AA162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="AB162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="AC162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
       <c r="AD162" t="n">
-        <v>477.6248999999999</v>
+        <v>477.625</v>
       </c>
     </row>
     <row r="163">
@@ -17530,76 +17530,76 @@
         </is>
       </c>
       <c r="G168" t="n">
-        <v>122.5008</v>
+        <v>122.501</v>
       </c>
       <c r="H168" t="n">
-        <v>122.5008</v>
+        <v>122.501</v>
       </c>
       <c r="I168" t="n">
-        <v>122.5008</v>
+        <v>122.501</v>
       </c>
       <c r="J168" t="n">
-        <v>122.5008</v>
+        <v>122.501</v>
       </c>
       <c r="K168" t="n">
-        <v>122.5008</v>
+        <v>122.501</v>
       </c>
       <c r="L168" t="n">
-        <v>122.5008</v>
+        <v>122.501</v>
       </c>
       <c r="M168" t="n">
-        <v>85.9248</v>
+        <v>85.925</v>
       </c>
       <c r="N168" t="n">
-        <v>85.9248</v>
+        <v>85.925</v>
       </c>
       <c r="O168" t="n">
-        <v>85.9248</v>
+        <v>85.925</v>
       </c>
       <c r="P168" t="n">
-        <v>85.9248</v>
+        <v>85.925</v>
       </c>
       <c r="Q168" t="n">
-        <v>85.9248</v>
+        <v>85.925</v>
       </c>
       <c r="R168" t="n">
-        <v>85.9248</v>
+        <v>85.925</v>
       </c>
       <c r="S168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="T168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="U168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="V168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="W168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="X168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="Y168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="Z168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="AA168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="AB168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="AC168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
       <c r="AD168" t="n">
-        <v>74.62480000000001</v>
+        <v>74.625</v>
       </c>
     </row>
     <row r="169">
@@ -17770,40 +17770,40 @@
         <v>56.977</v>
       </c>
       <c r="S170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="T170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="U170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="V170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="W170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="X170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="Y170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="Z170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="AA170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="AB170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="AC170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
       <c r="AD170" t="n">
-        <v>32.14400000000001</v>
+        <v>32.144</v>
       </c>
     </row>
     <row r="171">
@@ -17938,76 +17938,76 @@
         </is>
       </c>
       <c r="G172" t="n">
-        <v>51.91350829040319</v>
+        <v>51.914</v>
       </c>
       <c r="H172" t="n">
-        <v>51.91350829040319</v>
+        <v>51.914</v>
       </c>
       <c r="I172" t="n">
-        <v>51.91350829040319</v>
+        <v>51.914</v>
       </c>
       <c r="J172" t="n">
-        <v>51.91350829040319</v>
+        <v>51.914</v>
       </c>
       <c r="K172" t="n">
-        <v>51.91350829040319</v>
+        <v>51.914</v>
       </c>
       <c r="L172" t="n">
-        <v>51.91350829040319</v>
+        <v>51.914</v>
       </c>
       <c r="M172" t="n">
-        <v>50.91350829040319</v>
+        <v>50.914</v>
       </c>
       <c r="N172" t="n">
-        <v>50.91350829040319</v>
+        <v>50.914</v>
       </c>
       <c r="O172" t="n">
-        <v>50.91350829040319</v>
+        <v>50.914</v>
       </c>
       <c r="P172" t="n">
-        <v>50.91350829040319</v>
+        <v>50.914</v>
       </c>
       <c r="Q172" t="n">
-        <v>50.91350829040319</v>
+        <v>50.914</v>
       </c>
       <c r="R172" t="n">
-        <v>50.91350829040319</v>
+        <v>50.914</v>
       </c>
       <c r="S172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="T172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="U172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="V172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="W172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="X172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="Y172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="Z172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="AA172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="AB172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="AC172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
       <c r="AD172" t="n">
-        <v>55.31526869040317</v>
+        <v>55.315</v>
       </c>
     </row>
     <row r="173">
@@ -18142,76 +18142,76 @@
         </is>
       </c>
       <c r="G174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="H174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="I174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="J174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="K174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="L174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="M174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="N174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="O174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="P174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="Q174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="R174" t="n">
-        <v>109.7744917095968</v>
+        <v>109.774</v>
       </c>
       <c r="S174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="T174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="U174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="V174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="W174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="X174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="Y174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="Z174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="AA174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="AB174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="AC174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
       <c r="AD174" t="n">
-        <v>83.11473130959682</v>
+        <v>83.11499999999999</v>
       </c>
     </row>
     <row r="175">
@@ -19162,76 +19162,76 @@
         </is>
       </c>
       <c r="G184" t="n">
-        <v>4085.45378127909</v>
+        <v>4085.454</v>
       </c>
       <c r="H184" t="n">
-        <v>4085.45378127909</v>
+        <v>4085.454</v>
       </c>
       <c r="I184" t="n">
-        <v>4085.45378127909</v>
+        <v>4085.454</v>
       </c>
       <c r="J184" t="n">
-        <v>4085.45378127909</v>
+        <v>4085.454</v>
       </c>
       <c r="K184" t="n">
-        <v>4085.45378127909</v>
+        <v>4085.454</v>
       </c>
       <c r="L184" t="n">
-        <v>4085.45378127909</v>
+        <v>4085.454</v>
       </c>
       <c r="M184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="N184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="O184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="P184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="Q184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="R184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="S184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="T184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="U184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="V184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="W184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="X184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="Y184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="Z184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="AA184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="AB184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="AC184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
       <c r="AD184" t="n">
-        <v>4077.2007</v>
+        <v>4077.201</v>
       </c>
     </row>
     <row r="185">
@@ -20653,13 +20653,13 @@
         <v>126</v>
       </c>
       <c r="AB198" t="n">
-        <v>72.00000000000001</v>
+        <v>72</v>
       </c>
       <c r="AC198" t="n">
-        <v>72.00000000000001</v>
+        <v>72</v>
       </c>
       <c r="AD198" t="n">
-        <v>72.00000000000001</v>
+        <v>72</v>
       </c>
     </row>
     <row r="199">
@@ -27136,22 +27136,22 @@
         <v>114</v>
       </c>
       <c r="M262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="N262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="O262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="P262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="Q262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="R262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="S262" t="n">
         <v>49</v>
@@ -27172,22 +27172,22 @@
         <v>49</v>
       </c>
       <c r="Y262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="Z262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="AA262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="AB262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="AC262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
       <c r="AD262" t="n">
-        <v>1072.75264</v>
+        <v>1072.753</v>
       </c>
     </row>
     <row r="263">
@@ -30586,76 +30586,76 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="H296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="I296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="J296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="K296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="L296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="M296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="N296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="O296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="P296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="Q296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="R296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="S296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="T296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="U296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="V296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="W296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="X296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="Y296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="Z296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="AA296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="AB296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="AC296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
       <c r="AD296" t="n">
-        <v>25.8429</v>
+        <v>25.843</v>
       </c>
     </row>
     <row r="297">
@@ -32830,76 +32830,76 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="H318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="I318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="J318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="K318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="L318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="M318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="N318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="O318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="P318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="Q318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="R318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="S318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="T318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="U318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="V318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="W318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="X318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="Y318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="Z318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="AA318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="AB318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="AC318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
       <c r="AD318" t="n">
-        <v>468.0740799999999</v>
+        <v>468.074</v>
       </c>
     </row>
     <row r="319">
@@ -34666,76 +34666,76 @@
         </is>
       </c>
       <c r="G336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="H336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="I336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="J336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="K336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="L336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="M336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="N336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="O336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="P336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="Q336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="R336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="S336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="T336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="U336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="V336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="W336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="X336" t="n">
-        <v>2516.2206</v>
+        <v>2516.221</v>
       </c>
       <c r="Y336" t="n">
-        <v>2465.2206</v>
+        <v>2465.221</v>
       </c>
       <c r="Z336" t="n">
-        <v>2465.2206</v>
+        <v>2465.221</v>
       </c>
       <c r="AA336" t="n">
-        <v>2465.2206</v>
+        <v>2465.221</v>
       </c>
       <c r="AB336" t="n">
-        <v>2465.2206</v>
+        <v>2465.221</v>
       </c>
       <c r="AC336" t="n">
-        <v>2465.2206</v>
+        <v>2465.221</v>
       </c>
       <c r="AD336" t="n">
-        <v>2465.2206</v>
+        <v>2465.221</v>
       </c>
     </row>
     <row r="337">
@@ -37930,76 +37930,76 @@
         </is>
       </c>
       <c r="G368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="H368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="I368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="J368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="K368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="L368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="M368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="N368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="O368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="P368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="Q368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="R368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="S368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="T368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="U368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="V368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="W368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="X368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="Y368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="Z368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="AA368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="AB368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="AC368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
       <c r="AD368" t="n">
-        <v>224.53166</v>
+        <v>224.532</v>
       </c>
     </row>
     <row r="369">
@@ -39154,40 +39154,40 @@
         </is>
       </c>
       <c r="G380" t="n">
-        <v>9.688995215311005</v>
+        <v>9.689</v>
       </c>
       <c r="H380" t="n">
-        <v>9.688995215311005</v>
+        <v>9.689</v>
       </c>
       <c r="I380" t="n">
-        <v>9.688995215311005</v>
+        <v>9.689</v>
       </c>
       <c r="J380" t="n">
-        <v>9.688995215311005</v>
+        <v>9.689</v>
       </c>
       <c r="K380" t="n">
-        <v>9.688995215311005</v>
+        <v>9.689</v>
       </c>
       <c r="L380" t="n">
-        <v>9.688995215311005</v>
+        <v>9.689</v>
       </c>
       <c r="M380" t="n">
-        <v>6.45933014354067</v>
+        <v>6.459</v>
       </c>
       <c r="N380" t="n">
-        <v>6.45933014354067</v>
+        <v>6.459</v>
       </c>
       <c r="O380" t="n">
-        <v>6.45933014354067</v>
+        <v>6.459</v>
       </c>
       <c r="P380" t="n">
-        <v>6.45933014354067</v>
+        <v>6.459</v>
       </c>
       <c r="Q380" t="n">
-        <v>6.45933014354067</v>
+        <v>6.459</v>
       </c>
       <c r="R380" t="n">
-        <v>6.45933014354067</v>
+        <v>6.459</v>
       </c>
       <c r="S380" t="n">
         <v>0</v>
@@ -44068,22 +44068,22 @@
         <v>0</v>
       </c>
       <c r="M428" t="n">
-        <v>1709.242805870638</v>
+        <v>1709.243</v>
       </c>
       <c r="N428" t="n">
-        <v>1709.242805870638</v>
+        <v>1709.243</v>
       </c>
       <c r="O428" t="n">
-        <v>1709.242805870638</v>
+        <v>1709.243</v>
       </c>
       <c r="P428" t="n">
-        <v>1709.242805870638</v>
+        <v>1709.243</v>
       </c>
       <c r="Q428" t="n">
-        <v>1709.242805870638</v>
+        <v>1709.243</v>
       </c>
       <c r="R428" t="n">
-        <v>1709.242805870638</v>
+        <v>1709.243</v>
       </c>
       <c r="S428" t="n">
         <v>0</v>
@@ -44104,22 +44104,22 @@
         <v>0</v>
       </c>
       <c r="Y428" t="n">
-        <v>1758.618885870638</v>
+        <v>1758.619</v>
       </c>
       <c r="Z428" t="n">
-        <v>1758.618885870638</v>
+        <v>1758.619</v>
       </c>
       <c r="AA428" t="n">
-        <v>1758.618885870638</v>
+        <v>1758.619</v>
       </c>
       <c r="AB428" t="n">
-        <v>1758.618885870638</v>
+        <v>1758.619</v>
       </c>
       <c r="AC428" t="n">
-        <v>1758.618885870638</v>
+        <v>1758.619</v>
       </c>
       <c r="AD428" t="n">
-        <v>1758.618885870638</v>
+        <v>1758.619</v>
       </c>
     </row>
     <row r="429">
@@ -44272,22 +44272,22 @@
         <v>0</v>
       </c>
       <c r="M430" t="n">
-        <v>606.4468800000001</v>
+        <v>606.447</v>
       </c>
       <c r="N430" t="n">
-        <v>606.4468800000001</v>
+        <v>606.447</v>
       </c>
       <c r="O430" t="n">
-        <v>606.4468800000001</v>
+        <v>606.447</v>
       </c>
       <c r="P430" t="n">
-        <v>606.4468800000001</v>
+        <v>606.447</v>
       </c>
       <c r="Q430" t="n">
-        <v>606.4468800000001</v>
+        <v>606.447</v>
       </c>
       <c r="R430" t="n">
-        <v>606.4468800000001</v>
+        <v>606.447</v>
       </c>
       <c r="S430" t="n">
         <v>0</v>
@@ -44308,22 +44308,22 @@
         <v>0</v>
       </c>
       <c r="Y430" t="n">
-        <v>582.4808800000001</v>
+        <v>582.481</v>
       </c>
       <c r="Z430" t="n">
-        <v>582.4808800000001</v>
+        <v>582.481</v>
       </c>
       <c r="AA430" t="n">
-        <v>582.4808800000001</v>
+        <v>582.481</v>
       </c>
       <c r="AB430" t="n">
-        <v>582.4808800000001</v>
+        <v>582.481</v>
       </c>
       <c r="AC430" t="n">
-        <v>582.4808800000001</v>
+        <v>582.481</v>
       </c>
       <c r="AD430" t="n">
-        <v>582.4808800000001</v>
+        <v>582.481</v>
       </c>
     </row>
     <row r="431">
@@ -44662,40 +44662,40 @@
         </is>
       </c>
       <c r="G434" t="n">
-        <v>1984.6245</v>
+        <v>1984.624</v>
       </c>
       <c r="H434" t="n">
-        <v>1984.6245</v>
+        <v>1984.624</v>
       </c>
       <c r="I434" t="n">
-        <v>1984.6245</v>
+        <v>1984.624</v>
       </c>
       <c r="J434" t="n">
-        <v>1984.6245</v>
+        <v>1984.624</v>
       </c>
       <c r="K434" t="n">
-        <v>1984.6245</v>
+        <v>1984.624</v>
       </c>
       <c r="L434" t="n">
-        <v>1984.6245</v>
+        <v>1984.624</v>
       </c>
       <c r="M434" t="n">
-        <v>5100.76803089044</v>
+        <v>5100.768</v>
       </c>
       <c r="N434" t="n">
-        <v>5100.76803089044</v>
+        <v>5100.768</v>
       </c>
       <c r="O434" t="n">
-        <v>5100.76803089044</v>
+        <v>5100.768</v>
       </c>
       <c r="P434" t="n">
-        <v>5100.76803089044</v>
+        <v>5100.768</v>
       </c>
       <c r="Q434" t="n">
-        <v>5100.76803089044</v>
+        <v>5100.768</v>
       </c>
       <c r="R434" t="n">
-        <v>5100.76803089044</v>
+        <v>5100.768</v>
       </c>
       <c r="S434" t="n">
         <v>835</v>
@@ -44716,22 +44716,22 @@
         <v>835</v>
       </c>
       <c r="Y434" t="n">
-        <v>2361.74353089044</v>
+        <v>2361.744</v>
       </c>
       <c r="Z434" t="n">
-        <v>2361.74353089044</v>
+        <v>2361.744</v>
       </c>
       <c r="AA434" t="n">
-        <v>2361.74353089044</v>
+        <v>2361.744</v>
       </c>
       <c r="AB434" t="n">
-        <v>2361.74353089044</v>
+        <v>2361.744</v>
       </c>
       <c r="AC434" t="n">
-        <v>2361.74353089044</v>
+        <v>2361.744</v>
       </c>
       <c r="AD434" t="n">
-        <v>2361.74353089044</v>
+        <v>2361.744</v>
       </c>
     </row>
     <row r="435">
@@ -44866,40 +44866,40 @@
         </is>
       </c>
       <c r="G436" t="n">
-        <v>66.4755</v>
+        <v>66.47499999999999</v>
       </c>
       <c r="H436" t="n">
-        <v>66.4755</v>
+        <v>66.47499999999999</v>
       </c>
       <c r="I436" t="n">
-        <v>66.4755</v>
+        <v>66.47499999999999</v>
       </c>
       <c r="J436" t="n">
-        <v>66.4755</v>
+        <v>66.47499999999999</v>
       </c>
       <c r="K436" t="n">
-        <v>66.4755</v>
+        <v>66.47499999999999</v>
       </c>
       <c r="L436" t="n">
-        <v>66.4755</v>
+        <v>66.47499999999999</v>
       </c>
       <c r="M436" t="n">
-        <v>66.4755</v>
+        <v>66.47499999999999</v>
       </c>
       <c r="N436" t="n">
-        <v>66.4755</v>
+        <v>66.47499999999999</v>
       </c>
       <c r="O436" t="n">
-        <v>66.4755</v>
+        <v>66.47499999999999</v>
       </c>
       <c r="P436" t="n">
-        <v>66.4755</v>
+        <v>66.47499999999999</v>
       </c>
       <c r="Q436" t="n">
-        <v>66.4755</v>
+        <v>66.47499999999999</v>
       </c>
       <c r="R436" t="n">
-        <v>66.4755</v>
+        <v>66.47499999999999</v>
       </c>
       <c r="S436" t="n">
         <v>0</v>
@@ -45070,40 +45070,40 @@
         </is>
       </c>
       <c r="G438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="H438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="I438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="J438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="K438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="L438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="M438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="N438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="O438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="P438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="Q438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="R438" t="n">
-        <v>4442.872989392305</v>
+        <v>4442.873</v>
       </c>
       <c r="S438" t="n">
         <v>3670.75</v>
@@ -45274,58 +45274,58 @@
         </is>
       </c>
       <c r="G440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="H440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="I440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="J440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="K440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="L440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="M440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="N440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="O440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="P440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="Q440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="R440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="S440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="T440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="U440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="V440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="W440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="X440" t="n">
-        <v>560.2499999999999</v>
+        <v>560.25</v>
       </c>
       <c r="Y440" t="n">
         <v>0</v>
@@ -47548,7 +47548,7 @@
         <v>650</v>
       </c>
       <c r="Q462" t="n">
-        <v>1300</v>
+        <v>650</v>
       </c>
       <c r="R462" t="n">
         <v>1300</v>
@@ -47650,7 +47650,7 @@
         <v>1</v>
       </c>
       <c r="Q463" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R463" t="n">
         <v>2</v>
@@ -50170,76 +50170,76 @@
         </is>
       </c>
       <c r="G488" t="n">
-        <v>212.148282494181</v>
+        <v>212.148</v>
       </c>
       <c r="H488" t="n">
-        <v>212.148282494181</v>
+        <v>212.148</v>
       </c>
       <c r="I488" t="n">
-        <v>212.148282494181</v>
+        <v>212.148</v>
       </c>
       <c r="J488" t="n">
-        <v>212.148282494181</v>
+        <v>212.148</v>
       </c>
       <c r="K488" t="n">
-        <v>212.148282494181</v>
+        <v>212.148</v>
       </c>
       <c r="L488" t="n">
-        <v>218.5108942790641</v>
+        <v>212.148</v>
       </c>
       <c r="M488" t="n">
-        <v>218.5108942790641</v>
+        <v>218.511</v>
       </c>
       <c r="N488" t="n">
-        <v>218.5108942790641</v>
+        <v>218.511</v>
       </c>
       <c r="O488" t="n">
-        <v>218.5108942790641</v>
+        <v>218.511</v>
       </c>
       <c r="P488" t="n">
-        <v>218.5108942790641</v>
+        <v>218.511</v>
       </c>
       <c r="Q488" t="n">
-        <v>218.5108942790641</v>
+        <v>218.511</v>
       </c>
       <c r="R488" t="n">
-        <v>218.5108942790641</v>
+        <v>218.511</v>
       </c>
       <c r="S488" t="n">
-        <v>242.2384454244763</v>
+        <v>242.238</v>
       </c>
       <c r="T488" t="n">
-        <v>242.2384454244763</v>
+        <v>242.238</v>
       </c>
       <c r="U488" t="n">
-        <v>242.2384454244763</v>
+        <v>242.238</v>
       </c>
       <c r="V488" t="n">
-        <v>242.2384454244763</v>
+        <v>242.238</v>
       </c>
       <c r="W488" t="n">
-        <v>242.2384454244763</v>
+        <v>242.238</v>
       </c>
       <c r="X488" t="n">
-        <v>248.0267585446527</v>
+        <v>242.238</v>
       </c>
       <c r="Y488" t="n">
-        <v>248.0267585446527</v>
+        <v>248.027</v>
       </c>
       <c r="Z488" t="n">
-        <v>248.0267585446527</v>
+        <v>248.027</v>
       </c>
       <c r="AA488" t="n">
-        <v>248.0267585446527</v>
+        <v>248.027</v>
       </c>
       <c r="AB488" t="n">
-        <v>248.0267585446527</v>
+        <v>248.027</v>
       </c>
       <c r="AC488" t="n">
-        <v>248.0267585446527</v>
+        <v>248.027</v>
       </c>
       <c r="AD488" t="n">
-        <v>248.0267585446527</v>
+        <v>248.027</v>
       </c>
     </row>
     <row r="489">
@@ -50287,7 +50287,7 @@
         <v>13</v>
       </c>
       <c r="L489" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M489" t="n">
         <v>14</v>
@@ -50323,7 +50323,7 @@
         <v>18</v>
       </c>
       <c r="X489" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="Y489" t="n">
         <v>19</v>
@@ -51598,76 +51598,76 @@
         </is>
       </c>
       <c r="G502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="H502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="I502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="J502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="K502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="L502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="M502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="N502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="O502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="P502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="Q502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="R502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="S502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="T502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="U502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="V502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="W502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="X502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="Y502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="Z502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="AA502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="AB502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="AC502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
       <c r="AD502" t="n">
-        <v>85.55302610569625</v>
+        <v>85.553</v>
       </c>
     </row>
     <row r="503">
@@ -51802,76 +51802,76 @@
         </is>
       </c>
       <c r="G504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="H504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="I504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="J504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="K504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="L504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="M504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="N504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="O504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="P504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="Q504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="R504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="S504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="T504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="U504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="V504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="W504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="X504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="Y504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="Z504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="AA504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="AB504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="AC504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
       <c r="AD504" t="n">
-        <v>99.10897389430374</v>
+        <v>99.10899999999999</v>
       </c>
     </row>
     <row r="505">
@@ -52006,76 +52006,76 @@
         </is>
       </c>
       <c r="G506" t="n">
-        <v>120.8717305699482</v>
+        <v>120.872</v>
       </c>
       <c r="H506" t="n">
-        <v>120.8717305699482</v>
+        <v>120.872</v>
       </c>
       <c r="I506" t="n">
-        <v>120.8717305699482</v>
+        <v>120.872</v>
       </c>
       <c r="J506" t="n">
-        <v>120.8717305699482</v>
+        <v>120.872</v>
       </c>
       <c r="K506" t="n">
-        <v>120.8717305699482</v>
+        <v>120.872</v>
       </c>
       <c r="L506" t="n">
-        <v>120.8717305699482</v>
+        <v>120.872</v>
       </c>
       <c r="M506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="N506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="O506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="P506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="Q506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="R506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="S506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="T506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="U506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="V506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="W506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="X506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="Y506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="Z506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="AA506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="AB506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="AC506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
       <c r="AD506" t="n">
-        <v>124.8717305699482</v>
+        <v>124.872</v>
       </c>
     </row>
     <row r="507">
@@ -53026,76 +53026,76 @@
         </is>
       </c>
       <c r="G516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="H516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="I516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="J516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="K516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="L516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="M516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="N516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="O516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="P516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="Q516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="R516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="S516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="T516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="U516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="V516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="W516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="X516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="Y516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="Z516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="AA516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="AB516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="AC516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
       <c r="AD516" t="n">
-        <v>5.484712500000001</v>
+        <v>5.485</v>
       </c>
     </row>
     <row r="517">
@@ -53230,76 +53230,76 @@
         </is>
       </c>
       <c r="G518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="H518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="I518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="J518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="K518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="L518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="M518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="N518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="O518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="P518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="Q518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="R518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="S518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="T518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="U518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="V518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="W518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="X518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="Y518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="Z518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="AA518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="AB518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="AC518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
       <c r="AD518" t="n">
-        <v>21.6002875</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="519">
@@ -53638,76 +53638,76 @@
         </is>
       </c>
       <c r="G522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="H522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="I522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="J522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="K522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="L522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="M522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="N522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="O522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="P522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="Q522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="R522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="S522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="T522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="U522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="V522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="W522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="X522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="Y522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="Z522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="AA522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="AB522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="AC522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
       <c r="AD522" t="n">
-        <v>55.96109999999999</v>
+        <v>55.961</v>
       </c>
     </row>
     <row r="523">
@@ -53842,76 +53842,76 @@
         </is>
       </c>
       <c r="G524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="H524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="I524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="J524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="K524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="L524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="M524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="N524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="O524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="P524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="Q524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="R524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="S524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="T524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="U524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="V524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="W524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="X524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="Y524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="Z524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="AA524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="AB524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="AC524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
       <c r="AD524" t="n">
-        <v>10.4139</v>
+        <v>10.414</v>
       </c>
     </row>
     <row r="525">
@@ -54250,76 +54250,76 @@
         </is>
       </c>
       <c r="G528" t="n">
-        <v>2789.137264415848</v>
+        <v>2789.137</v>
       </c>
       <c r="H528" t="n">
-        <v>2789.137264415848</v>
+        <v>2789.137</v>
       </c>
       <c r="I528" t="n">
-        <v>2789.137264415848</v>
+        <v>2789.137</v>
       </c>
       <c r="J528" t="n">
-        <v>2789.137264415848</v>
+        <v>2789.137</v>
       </c>
       <c r="K528" t="n">
-        <v>2789.137264415848</v>
+        <v>2789.137</v>
       </c>
       <c r="L528" t="n">
-        <v>2789.137264415848</v>
+        <v>2789.137</v>
       </c>
       <c r="M528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="N528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="O528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="P528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="Q528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="R528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="S528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="T528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="U528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="V528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="W528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="X528" t="n">
-        <v>2814.637264415849</v>
+        <v>2814.637</v>
       </c>
       <c r="Y528" t="n">
-        <v>2829.637264415848</v>
+        <v>2829.637</v>
       </c>
       <c r="Z528" t="n">
-        <v>2829.637264415848</v>
+        <v>2829.637</v>
       </c>
       <c r="AA528" t="n">
-        <v>2829.637264415848</v>
+        <v>2829.637</v>
       </c>
       <c r="AB528" t="n">
-        <v>2829.637264415848</v>
+        <v>2829.637</v>
       </c>
       <c r="AC528" t="n">
-        <v>2829.637264415848</v>
+        <v>2829.637</v>
       </c>
       <c r="AD528" t="n">
-        <v>2829.637264415848</v>
+        <v>2829.637</v>
       </c>
     </row>
     <row r="529">
@@ -55120,22 +55120,22 @@
         <v>1612.71</v>
       </c>
       <c r="Y536" t="n">
-        <v>851.0699999999999</v>
+        <v>851.0700000000001</v>
       </c>
       <c r="Z536" t="n">
-        <v>851.0699999999999</v>
+        <v>851.0700000000001</v>
       </c>
       <c r="AA536" t="n">
-        <v>851.0699999999999</v>
+        <v>851.0700000000001</v>
       </c>
       <c r="AB536" t="n">
-        <v>851.0699999999999</v>
+        <v>851.0700000000001</v>
       </c>
       <c r="AC536" t="n">
-        <v>851.0699999999999</v>
+        <v>851.0700000000001</v>
       </c>
       <c r="AD536" t="n">
-        <v>851.0699999999999</v>
+        <v>851.0700000000001</v>
       </c>
     </row>
     <row r="537">

</xml_diff>